<commit_message>
complete mlp, cv, hp tuning, calibration, summary improved
</commit_message>
<xml_diff>
--- a/results/performance_summary.xlsx
+++ b/results/performance_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,12 +458,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>555.31%</t>
+          <t>158878.16%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>426.97%</t>
+          <t>76442.90%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,12 +485,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>60.22%</t>
+          <t>534.93%</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>51.70%</t>
+          <t>428.60%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -512,12 +512,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>27.45%</t>
+          <t>28.31%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27.41%</t>
+          <t>28.18%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -534,73 +534,81 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Sharpe Ratio</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1.89</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.88</v>
+          <t>Semi-volatility</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>15.06%</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>15.26%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>11.73%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>14.72%</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Minimum Return</t>
+          <t>Sharpe Ratio</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-6.27%</t>
+          <t>18.90</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-6.46%</t>
+          <t>15.21</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-5.14%</t>
+          <t>0.88</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Maximum Return</t>
+          <t>Sortino Ratio</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6.13%</t>
+          <t>35.52</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6.10%</t>
+          <t>28.08</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>1.34</t>
         </is>
       </c>
     </row>
@@ -612,12 +620,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-20.69%</t>
+          <t>-9.46%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-23.13%</t>
+          <t>-10.81%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -634,27 +642,27 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Value at Risk (VaR)</t>
+          <t>Avg Drawdown</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-2.53%</t>
+          <t>-1.10%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-2.55%</t>
+          <t>-1.29%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.66%</t>
+          <t>-6.12%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-2.29%</t>
+          <t>-7.13%</t>
         </is>
       </c>
     </row>
@@ -666,12 +674,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>-3.74%</t>
+          <t>-2.87%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-3.79%</t>
+          <t>-2.96%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -688,108 +696,180 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Trade Count</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2276</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2276</v>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+          <t>Skew</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.297</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.264</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-0.204</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-0.188</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Win Rate</t>
+          <t>Kurtosis</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>39.94%</t>
+          <t>0.385</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>39.94%</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+          <t>0.405</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1.927</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.652</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Turnover</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>218.6310493830005</v>
-      </c>
-      <c r="C13" t="n">
-        <v>218.6310493830005</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+          <t>Correlation to SPY</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-0.011</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-0.009</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0.825</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>TP Trades</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>909</v>
-      </c>
-      <c r="C14" t="n">
-        <v>909</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+          <t>Std Dev Correlation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0.479</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0.479</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0.113</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>SL Trades</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1367</v>
-      </c>
-      <c r="C15" t="n">
-        <v>1367</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1.897</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1.712</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-0.000</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.048</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Time Barrier Trades</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3010</v>
-      </c>
-      <c r="C16" t="n">
-        <v>3010</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>-0.019</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>-0.016</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.118</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Avg Holding Period (days)</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>7.33</v>
-      </c>
-      <c r="C17" t="n">
-        <v>7.33</v>
+          <t>Avg Leverage (Gross)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1.91</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1.91</t>
+        </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
@@ -797,17 +877,17 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Avg PnL per Trade</t>
+          <t>Max Leverage (Gross)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.24%</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.19%</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -816,21 +896,268 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Exposure-Weighted Win Rate</t>
+          <t>Avg Net Exposure</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>-0.14</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17.09%</t>
+          <t>-0.14</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Trade Count</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>8347</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8347</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Win Rate</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>62.20%</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>62.20%</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Avg Daily Turnover</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>TP Trades</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1865</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1865</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>SL Trades</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2328</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2328</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Timeout / No Signal</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4154</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>4154</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Avg Holding Period (days)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>11.58</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>11.58</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Notional-Weighted Win Rate</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>60.47%</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>60.47%</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Avg PnL per Trade</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0.26%</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0.26%</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Median PnL per Trade</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0.11%</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0.11%</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2.39</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2.39</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Long Hit Rate</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>22.34%</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>22.34%</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>Short Hit Rate</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Main: stable stack only (experimental paths removed)
</commit_message>
<xml_diff>
--- a/results/performance_summary.xlsx
+++ b/results/performance_summary.xlsx
@@ -473,22 +473,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>9.15%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>3.60%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>10.22%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5.09%</t>
+          <t>6.06%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -515,22 +515,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20.01%</t>
+          <t>19.59%</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>20.02%</t>
+          <t>19.60%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13.27%</t>
+          <t>13.19%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>19.75%</t>
+          <t>19.35%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -557,22 +557,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>15.90%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>16.71%</t>
+          <t>15.87%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>10.13%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>16.33%</t>
+          <t>15.49%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -599,22 +599,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -641,22 +641,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.58</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.39</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -683,22 +683,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-3.14%</t>
+          <t>-3.02%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-3.16%</t>
+          <t>-3.04%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-1.97%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-2.99%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -725,22 +725,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-32.13%</t>
+          <t>-27.90%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-33.16%</t>
+          <t>-29.83%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-30.33%</t>
+          <t>-28.45%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-36.30%</t>
+          <t>-32.05%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -767,22 +767,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-10.38%</t>
+          <t>-8.53%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-13.57%</t>
+          <t>-11.42%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-4.25%</t>
+          <t>-3.96%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-11.65%</t>
+          <t>-9.81%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -809,22 +809,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>452</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>492</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>512</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>193</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -851,22 +851,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>-1.091</t>
+          <t>-0.846</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-1.093</t>
+          <t>-0.847</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.781</t>
+          <t>-0.650</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-1.151</t>
+          <t>-0.899</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -893,22 +893,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.721</t>
+          <t>7.814</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10.698</t>
+          <t>7.801</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6.375</t>
+          <t>5.141</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9.330</t>
+          <t>6.674</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -935,22 +935,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-0.163</t>
+          <t>-0.157</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-0.162</t>
+          <t>-0.156</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.668</t>
+          <t>0.680</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -977,22 +977,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.122</t>
+          <t>0.130</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.069</t>
+          <t>0.078</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.035</t>
+          <t>0.039</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.069</t>
+          <t>0.078</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1019,22 +1019,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-0.156</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-0.155</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.423</t>
+          <t>0.427</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1061,22 +1061,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>34</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>34</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>33</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1103,22 +1103,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>25</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>26</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>27</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5724</t>
+          <t>5672</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5724</t>
+          <t>5672</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>61.69%</t>
+          <t>60.54%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>61.69%</t>
+          <t>60.54%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3071</t>
+          <t>3076</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3071</t>
+          <t>3076</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1964</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1964</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>645</t>
+          <t>632</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>645</t>
+          <t>632</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>24.97</t>
+          <t>25.97</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>24.97</t>
+          <t>25.97</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>62.24%</t>
+          <t>60.15%</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>62.24%</t>
+          <t>60.15%</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.22%</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>55.06%</t>
+          <t>56.18%</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>55.06%</t>
+          <t>56.18%</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>48.98%</t>
+          <t>47.43%</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>48.98%</t>
+          <t>47.43%</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>

<commit_message>
small bug fix, same in main
</commit_message>
<xml_diff>
--- a/results/performance_summary.xlsx
+++ b/results/performance_summary.xlsx
@@ -473,22 +473,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8.01%</t>
+          <t>16.74%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>12.17%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9.67%</t>
+          <t>14.64%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5.09%</t>
+          <t>14.20%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -515,22 +515,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20.01%</t>
+          <t>19.50%</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>20.02%</t>
+          <t>19.51%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13.27%</t>
+          <t>13.43%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>19.75%</t>
+          <t>19.36%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -557,22 +557,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.75%</t>
+          <t>15.14%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>16.71%</t>
+          <t>15.13%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.37%</t>
+          <t>10.17%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>16.33%</t>
+          <t>14.92%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -599,22 +599,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>0.86</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>0.73</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -641,22 +641,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -683,22 +683,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-3.14%</t>
+          <t>-2.95%</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-3.16%</t>
+          <t>-2.97%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-1.99%</t>
+          <t>-2.00%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-3.11%</t>
+          <t>-2.94%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -725,22 +725,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-32.13%</t>
+          <t>-27.32%</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-33.16%</t>
+          <t>-28.07%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-30.33%</t>
+          <t>-28.07%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-36.30%</t>
+          <t>-30.60%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -767,22 +767,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-10.38%</t>
+          <t>-6.07%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-13.57%</t>
+          <t>-7.05%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-4.25%</t>
+          <t>-4.14%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-11.65%</t>
+          <t>-6.82%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -809,22 +809,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>297</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>305</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>211</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>301</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -851,22 +851,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>-1.091</t>
+          <t>-0.700</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-1.093</t>
+          <t>-0.702</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.781</t>
+          <t>-0.553</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-1.151</t>
+          <t>-0.729</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -893,22 +893,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10.721</t>
+          <t>4.657</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10.698</t>
+          <t>4.647</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6.375</t>
+          <t>3.803</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9.330</t>
+          <t>4.147</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -935,17 +935,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-0.163</t>
+          <t>-0.122</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-0.162</t>
+          <t>-0.121</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.668</t>
+          <t>0.693</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -977,22 +977,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.122</t>
+          <t>0.192</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.069</t>
+          <t>0.152</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.035</t>
+          <t>0.076</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.069</t>
+          <t>0.152</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1019,17 +1019,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-0.156</t>
+          <t>-0.113</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-0.155</t>
+          <t>-0.113</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.423</t>
+          <t>0.444</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1061,22 +1061,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>38</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>38</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1103,22 +1103,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5724</t>
+          <t>3612</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5724</t>
+          <t>3612</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>61.69%</t>
+          <t>65.75%</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>61.69%</t>
+          <t>65.75%</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3071</t>
+          <t>2078</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3071</t>
+          <t>2078</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1145</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1145</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>645</t>
+          <t>389</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>645</t>
+          <t>389</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>24.97</t>
+          <t>24.2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>24.97</t>
+          <t>24.2</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>62.24%</t>
+          <t>65.81%</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>62.24%</t>
+          <t>65.81%</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.84%</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.33%</t>
+          <t>0.84%</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.38%</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.23%</t>
+          <t>0.38%</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>55.06%</t>
+          <t>57.43%</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>55.06%</t>
+          <t>57.43%</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>48.98%</t>
+          <t>61.29%</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>48.98%</t>
+          <t>61.29%</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>